<commit_message>
feat(candidate): implement create candidate with transaction, get candidate by id, new database schema, optimize image file manager code
</commit_message>
<xml_diff>
--- a/Modules.xlsx
+++ b/Modules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\GLP.Basecode.API.Voting\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gian Lloyd\Documents\GitHub\GLP.Basecode.API.Voting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93800B7A-6C24-4E38-965C-D5D4BBF71671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CEDEC5-4CA6-4E43-B489-FF2DD1704783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" xr2:uid="{631B70AB-E6AF-41D8-A199-357B3A98B252}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{631B70AB-E6AF-41D8-A199-357B3A98B252}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
   <si>
     <t>Modules</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>Generate a pdf file for the candidates details along with their number of votes.</t>
+  </si>
+  <si>
+    <t>Not testet</t>
   </si>
 </sst>
 </file>
@@ -575,11 +578,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{402DA261-852C-4A23-BAFF-35C124DBF4B2}">
-  <dimension ref="A2:Q31"/>
+  <dimension ref="A2:R31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="35.140625" customWidth="1"/>
+    <col min="18" max="18" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -890,7 +894,7 @@
       <c r="O16" s="5"/>
       <c r="P16" s="5"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>27</v>
       </c>
@@ -911,7 +915,7 @@
       <c r="O17" s="5"/>
       <c r="P17" s="5"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -938,7 +942,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>33</v>
       </c>
@@ -962,7 +966,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -985,8 +989,14 @@
       <c r="N20" s="5"/>
       <c r="O20" s="5"/>
       <c r="P20" s="5"/>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>45</v>
       </c>
@@ -1007,7 +1017,7 @@
       <c r="O21" s="5"/>
       <c r="P21" s="5"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>48</v>
       </c>
@@ -1028,7 +1038,7 @@
       <c r="O22" s="5"/>
       <c r="P22" s="5"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>50</v>
       </c>
@@ -1052,7 +1062,7 @@
       <c r="O23" s="5"/>
       <c r="P23" s="5"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
@@ -1076,7 +1086,7 @@
       <c r="O24" s="5"/>
       <c r="P24" s="5"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -1093,7 +1103,7 @@
       <c r="O25" s="5"/>
       <c r="P25" s="5"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
@@ -1109,7 +1119,7 @@
       <c r="O26" s="5"/>
       <c r="P26" s="5"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
@@ -1125,7 +1135,7 @@
       <c r="O27" s="5"/>
       <c r="P27" s="5"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
@@ -1141,7 +1151,7 @@
       <c r="O28" s="5"/>
       <c r="P28" s="5"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -1157,7 +1167,7 @@
       <c r="O29" s="5"/>
       <c r="P29" s="5"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
@@ -1173,7 +1183,7 @@
       <c r="O30" s="5"/>
       <c r="P30" s="5"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
@@ -1191,6 +1201,18 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="C31:P31"/>
+    <mergeCell ref="C23:P23"/>
+    <mergeCell ref="C24:P24"/>
+    <mergeCell ref="C25:P25"/>
+    <mergeCell ref="C26:P26"/>
+    <mergeCell ref="C27:P27"/>
+    <mergeCell ref="C28:P28"/>
+    <mergeCell ref="C18:P18"/>
+    <mergeCell ref="C20:P20"/>
+    <mergeCell ref="C21:P21"/>
+    <mergeCell ref="C29:P29"/>
+    <mergeCell ref="C30:P30"/>
     <mergeCell ref="C22:P22"/>
     <mergeCell ref="C14:P14"/>
     <mergeCell ref="C4:P4"/>
@@ -1207,18 +1229,6 @@
     <mergeCell ref="C5:P5"/>
     <mergeCell ref="C17:P17"/>
     <mergeCell ref="C19:P19"/>
-    <mergeCell ref="C18:P18"/>
-    <mergeCell ref="C20:P20"/>
-    <mergeCell ref="C21:P21"/>
-    <mergeCell ref="C29:P29"/>
-    <mergeCell ref="C30:P30"/>
-    <mergeCell ref="C31:P31"/>
-    <mergeCell ref="C23:P23"/>
-    <mergeCell ref="C24:P24"/>
-    <mergeCell ref="C25:P25"/>
-    <mergeCell ref="C26:P26"/>
-    <mergeCell ref="C27:P27"/>
-    <mergeCell ref="C28:P28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>